<commit_message>
New 4.0.5 files, temp using US
</commit_message>
<xml_diff>
--- a/InputData/web-app/CID/Check Input Data.xlsx
+++ b/InputData/web-app/CID/Check Input Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\web-app\CID\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163C0356-9559-4EF1-91ED-80F67B681CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23430FE0-5759-4E08-B06F-388D855B8D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="3" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -110,9 +110,6 @@
     <t>elec/BDTPTUMCF/BDTPTUMCF.csv</t>
   </si>
   <si>
-    <t>elec/RQSD/RQSD-BRQSD.csv</t>
-  </si>
-  <si>
     <t>elec/RQSD/RQSD-RQSD.csv</t>
   </si>
   <si>
@@ -131,12 +128,6 @@
     <t>trans/VTStFES/VTStFES.csv</t>
   </si>
   <si>
-    <t>elec/ESUfRaLCD/ESUfRaLCD-dispatch.csv</t>
-  </si>
-  <si>
-    <t>elec/ESUfRaLCD/ESUfRaLCD-reliability.csv</t>
-  </si>
-  <si>
     <t>plcy-schd/FoPITY/FoPITY-policy-elements.csv</t>
   </si>
   <si>
@@ -186,6 +177,15 @@
   </si>
   <si>
     <t>trans/VTQaZ/VTQaZ-motorbikes.csv</t>
+  </si>
+  <si>
+    <t>elec/RQSD/RQSD-CQSD.csv</t>
+  </si>
+  <si>
+    <t>ctrl-settings/BEEEfEPS/BEEEfEPS.csv</t>
+  </si>
+  <si>
+    <t>ctrl-settings/MV/MV-historical.csv</t>
   </si>
 </sst>
 </file>
@@ -572,18 +572,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB40378-4D92-6B46-95EC-BF41FEF6A51A}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.09765625" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="2"/>
+    <col min="1" max="1" width="15.06640625" style="2" customWidth="1"/>
+    <col min="2" max="16384" width="10.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -591,14 +591,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -609,55 +609,55 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD815B91-4D8D-3140-B01A-98F4799EC5EA}">
   <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="1"/>
+    <col min="1" max="1" width="20.265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -667,179 +667,178 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15C2FCA3-2250-8E45-A26E-181733CE1D14}">
-  <dimension ref="A1:A38"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A33"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="32.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="1"/>
+    <col min="1" max="1" width="32.06640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -847,210 +846,34 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176A5F9D-06D4-2548-AA03-82624CE63230}">
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="1"/>
+    <col min="2" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
-    <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="40f4d404-d193-41dc-bb72-733c1e774208" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC7782A9-2002-411F-B137-CBBBF6F81661}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A998D11-D0E9-47E7-8F9F-E4A9F5AFB9D8}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407C7143-C55C-4E8E-8D83-065FA303CDFE}"/>
 </file>
</xml_diff>